<commit_message>
refactor: :art: add DDD folder structure; changed the claims engine structure
</commit_message>
<xml_diff>
--- a/inputs/ri_outward.xlsx
+++ b/inputs/ri_outward.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://barentsreinsurance-my.sharepoint.com/personal/erik_pillon_barentsre_eu/Documents/Desktop/Azure/reserving-tools/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{1BEDFA60-B779-42E9-A45A-ECD607B9C26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A91EBD3D-B114-490B-8D68-909B192BEDBB}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{1BEDFA60-B779-42E9-A45A-ECD607B9C26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8694C72B-5558-4477-A1D8-E5F410B2DFF0}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="1008" windowWidth="30912" windowHeight="15288" xr2:uid="{0A157EF3-62A8-4227-AF72-AB2727612FB5}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15285" activeTab="2" xr2:uid="{0A157EF3-62A8-4227-AF72-AB2727612FB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Energy" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
-    <sheet name="Property" sheetId="1" r:id="rId3"/>
+    <sheet name="Property_Risk" sheetId="1" r:id="rId2"/>
+    <sheet name="Property_Cat" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,14 +38,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="21">
   <si>
     <t>n_reinstatements</t>
   </si>
   <si>
-    <t>layer_number</t>
-  </si>
-  <si>
     <t>limit</t>
   </si>
   <si>
@@ -92,6 +89,18 @@
   </si>
   <si>
     <t>layer_name</t>
+  </si>
+  <si>
+    <t>external_QS</t>
+  </si>
+  <si>
+    <t>layer_type</t>
+  </si>
+  <si>
+    <t>XoL</t>
+  </si>
+  <si>
+    <t>Proportional</t>
   </si>
 </sst>
 </file>
@@ -485,47 +494,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9774F855-4AA4-43B3-8D8F-D2F51795282C}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
       </c>
       <c r="B2">
         <v>5000000</v>
@@ -548,10 +560,13 @@
       <c r="H2">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>20000000</v>
@@ -571,10 +586,13 @@
       <c r="H3">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>25000000</v>
@@ -594,10 +612,13 @@
       <c r="H4">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>30000000</v>
@@ -617,10 +638,13 @@
       <c r="H5">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>7500000</v>
@@ -643,10 +667,13 @@
       <c r="H6">
         <v>0.125</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>12500000</v>
@@ -666,10 +693,13 @@
       <c r="H7">
         <v>0.125</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>20000000</v>
@@ -689,10 +719,13 @@
       <c r="H8">
         <v>0.125</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>20000000</v>
@@ -712,10 +745,13 @@
       <c r="H9">
         <v>0.125</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>20000000</v>
@@ -734,6 +770,29 @@
       </c>
       <c r="H10">
         <v>0.125</v>
+      </c>
+      <c r="I10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11">
+        <v>90000000</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0.25</v>
+      </c>
+      <c r="I11" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -754,290 +813,238 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCD9C08A-1198-4BEB-8037-14539C395C39}">
-  <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44236211-C8BC-42D8-A0F5-4219F1B388AE}">
+  <sheetPr codeName="Sheet3"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
       <c r="B2">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="C2">
-        <v>10000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2">
-        <v>5000000</v>
-      </c>
-      <c r="E2" s="2">
-        <v>2</v>
-      </c>
-      <c r="F2" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.34499999999999997</v>
+        <v>0.25</v>
       </c>
       <c r="H2">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>20000000</v>
+        <v>3000000</v>
       </c>
       <c r="C3">
-        <v>15000000</v>
-      </c>
-      <c r="E3" s="2">
-        <v>2</v>
-      </c>
-      <c r="F3" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>0.36</v>
+        <v>0.15</v>
       </c>
       <c r="H3">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>25000000</v>
-      </c>
-      <c r="C4">
-        <v>35000000</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>0.24</v>
-      </c>
-      <c r="H4">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>30000000</v>
-      </c>
-      <c r="C5">
-        <v>60000000</v>
-      </c>
-      <c r="E5" s="2">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>0.11749999999999999</v>
-      </c>
-      <c r="H5">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>7500000</v>
-      </c>
-      <c r="C6">
-        <v>10000000</v>
-      </c>
-      <c r="D6">
-        <v>2500000</v>
-      </c>
-      <c r="E6" s="2">
-        <v>2</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>0.4</v>
-      </c>
-      <c r="H6">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7">
-        <v>12500000</v>
-      </c>
-      <c r="C7">
-        <v>17500000</v>
-      </c>
-      <c r="E7" s="2">
-        <v>2</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1</v>
-      </c>
-      <c r="G7">
-        <v>0.35</v>
-      </c>
-      <c r="H7">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>3</v>
-      </c>
-      <c r="B8">
-        <v>20000000</v>
-      </c>
-      <c r="C8">
-        <v>30000000</v>
-      </c>
-      <c r="E8" s="2">
-        <v>1</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1</v>
-      </c>
-      <c r="G8">
-        <v>0.27500000000000002</v>
-      </c>
-      <c r="H8">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>4</v>
-      </c>
-      <c r="B9">
-        <v>20000000</v>
-      </c>
-      <c r="C9">
-        <v>50000000</v>
-      </c>
-      <c r="E9" s="2">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3">
-        <v>1</v>
-      </c>
-      <c r="G9">
-        <v>0.18</v>
-      </c>
-      <c r="H9">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>5</v>
-      </c>
-      <c r="B10">
-        <v>20000000</v>
-      </c>
-      <c r="C10">
-        <v>70000000</v>
-      </c>
-      <c r="E10" s="2">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>0.11</v>
-      </c>
-      <c r="H10">
-        <v>0.125</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E4" s="2"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E5" s="2"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E6" s="2"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E7" s="2"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E8" s="2"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E9" s="2"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E10" s="2"/>
+      <c r="F10" s="3"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" display="mailto:1@100%25" xr:uid="{53E7C637-5DD0-4C5E-B0B0-580B44991895}"/>
-    <hyperlink ref="E5" r:id="rId2" display="mailto:1@100%25" xr:uid="{8C0B71D6-2A61-4FBC-BCA0-7134B029614E}"/>
-    <hyperlink ref="E8" r:id="rId3" display="mailto:1@100%25" xr:uid="{17AABD6C-BD5F-4EBE-8944-3229998CE965}"/>
-    <hyperlink ref="E9" r:id="rId4" display="mailto:1@100%25" xr:uid="{9B139E7C-C6D8-41AD-9B56-67E6DB940CE3}"/>
-    <hyperlink ref="E10" r:id="rId5" display="mailto:1@100%25" xr:uid="{B87AC1C9-7074-4934-9AE5-FD384D247C4A}"/>
-    <hyperlink ref="F4" r:id="rId6" display="mailto:1@100%25" xr:uid="{BFA49EB8-4B05-4B99-A0D7-2A3B20E71AD7}"/>
-    <hyperlink ref="F5" r:id="rId7" display="mailto:1@100%25" xr:uid="{773A8FEC-B22C-483F-9FE8-4DD56C14C776}"/>
-    <hyperlink ref="F8" r:id="rId8" display="mailto:1@100%25" xr:uid="{8DD443AD-1E28-4F0C-9A8D-DCDAE0DA98A5}"/>
-    <hyperlink ref="F9" r:id="rId9" display="mailto:1@100%25" xr:uid="{07DD83E8-B4C2-4E53-8C82-2AF13C0CAA29}"/>
-    <hyperlink ref="F10" r:id="rId10" display="mailto:1@100%25" xr:uid="{15732062-4B55-42D0-AA83-B9FC05665D47}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44236211-C8BC-42D8-A0F5-4219F1B388AE}">
-  <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD58421-85AF-4425-8A61-76C65378840F}">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>6000000</v>
+      </c>
+      <c r="C2">
+        <v>3000000</v>
+      </c>
+      <c r="D2">
+        <v>1000000</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0.24</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E3" s="2"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E4" s="2"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E5" s="2"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E6" s="2"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E7" s="2"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E8" s="2"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E9" s="2"/>
+      <c r="F9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor: :art: improved reinstatement premiums calculation for proportional Layers
</commit_message>
<xml_diff>
--- a/inputs/ri_outward.xlsx
+++ b/inputs/ri_outward.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://barentsreinsurance-my.sharepoint.com/personal/erik_pillon_barentsre_eu/Documents/Desktop/Azure/reserving-tools/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="8_{1BEDFA60-B779-42E9-A45A-ECD607B9C26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8694C72B-5558-4477-A1D8-E5F410B2DFF0}"/>
+  <xr:revisionPtr revIDLastSave="144" documentId="8_{1BEDFA60-B779-42E9-A45A-ECD607B9C26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3A79717-07E4-414F-93D0-FF149349FF35}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15285" activeTab="2" xr2:uid="{0A157EF3-62A8-4227-AF72-AB2727612FB5}"/>
+    <workbookView xWindow="-132" yWindow="-132" windowWidth="30984" windowHeight="16824" xr2:uid="{0A157EF3-62A8-4227-AF72-AB2727612FB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Energy" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="22">
   <si>
     <t>n_reinstatements</t>
   </si>
@@ -101,6 +101,9 @@
   </si>
   <si>
     <t>Proportional</t>
+  </si>
+  <si>
+    <t>internal_QS</t>
   </si>
 </sst>
 </file>
@@ -494,19 +497,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9774F855-4AA4-43B3-8D8F-D2F51795282C}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -535,7 +538,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -564,7 +567,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -590,7 +593,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -616,7 +619,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -642,7 +645,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -671,7 +674,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -697,7 +700,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -723,7 +726,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -749,7 +752,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -775,7 +778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -785,13 +788,27 @@
       <c r="C11">
         <v>0</v>
       </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
       <c r="H11">
         <v>0.25</v>
       </c>
       <c r="I11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12">
+        <v>90000000</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0.9</v>
+      </c>
+      <c r="I12" t="s">
         <v>20</v>
       </c>
     </row>
@@ -816,19 +833,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44236211-C8BC-42D8-A0F5-4219F1B388AE}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -857,7 +874,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -886,7 +903,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -912,31 +929,31 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E4" s="2"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E5" s="2"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E10" s="2"/>
       <c r="F10" s="3"/>
     </row>
@@ -948,19 +965,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD58421-85AF-4425-8A61-76C65378840F}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -989,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1018,31 +1035,31 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E3" s="2"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E4" s="2"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E5" s="2"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
     </row>

</xml_diff>